<commit_message>
Timothy/Added search bar in edit, scroll for editing shifts
</commit_message>
<xml_diff>
--- a/data/staff_data.xlsx
+++ b/data/staff_data.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shifts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -399,7 +400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -421,6 +422,21 @@
           <t>Role</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Day  </t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> End Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -442,4 +458,238 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>01:03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>02:03</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Timothy/Fixed Calling Eclat Model from frontend
</commit_message>
<xml_diff>
--- a/data/staff_data.xlsx
+++ b/data/staff_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/616305462e2c924d/Desktop/UWB-Hackathon-2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_4DEBD679E6A73CF3BCA26B010E727A39F5503CB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02E13052-1D1E-44E5-ACEE-2FED006F5081}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_316B4BB6A285A0F2BBE6C7020EABCC17DDA02B9D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17160" yWindow="2715" windowWidth="9795" windowHeight="8415" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Staff" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
   <si>
     <t>Full Name</t>
   </si>
@@ -32,42 +32,63 @@
     <t>Role</t>
   </si>
   <si>
+    <t>osm_id</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>mike</t>
+  </si>
+  <si>
+    <t>mike@gmail.com</t>
+  </si>
+  <si>
+    <t>eployee</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>john@email.com</t>
+  </si>
+  <si>
+    <t>cook</t>
+  </si>
+  <si>
+    <t>jacjac</t>
+  </si>
+  <si>
+    <t>jac@maail</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>mat</t>
+  </si>
+  <si>
+    <t>maw@gmail</t>
+  </si>
+  <si>
+    <t>blob</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
     <t>Start Time</t>
   </si>
   <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>test@gmail.com</t>
-  </si>
-  <si>
-    <t>Manager</t>
-  </si>
-  <si>
-    <t>mike</t>
-  </si>
-  <si>
-    <t>mike@gmail.com</t>
-  </si>
-  <si>
-    <t>eployee</t>
-  </si>
-  <si>
-    <t>john</t>
-  </si>
-  <si>
-    <t>john@email.com</t>
-  </si>
-  <si>
-    <t>cook</t>
-  </si>
-  <si>
-    <t>Employee</t>
-  </si>
-  <si>
-    <t>Day</t>
-  </si>
-  <si>
     <t>End Time</t>
   </si>
   <si>
@@ -77,46 +98,34 @@
     <t>03:00</t>
   </si>
   <si>
-    <t>11:20</t>
+    <t>22:00</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>23:00</t>
+  </si>
+  <si>
+    <t>03:01</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>03:02</t>
+  </si>
+  <si>
+    <t>13:10</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
   </si>
   <si>
     <t>Wednesday</t>
-  </si>
-  <si>
-    <t>01:03</t>
-  </si>
-  <si>
-    <t>02:03</t>
-  </si>
-  <si>
-    <t>Tuesday</t>
-  </si>
-  <si>
-    <t>Thursday</t>
-  </si>
-  <si>
-    <t>Friday</t>
-  </si>
-  <si>
-    <t>Saturday</t>
-  </si>
-  <si>
-    <t>Sunday</t>
-  </si>
-  <si>
-    <t>22:00</t>
-  </si>
-  <si>
-    <t>23:00</t>
-  </si>
-  <si>
-    <t>03:01</t>
-  </si>
-  <si>
-    <t>03:02</t>
-  </si>
-  <si>
-    <t>13:10</t>
   </si>
 </sst>
 </file>
@@ -443,13 +452,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -459,8 +469,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -470,8 +483,11 @@
       <c r="C2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>11476372224</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -481,8 +497,11 @@
       <c r="C3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>11476372224</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -491,6 +510,37 @@
       </c>
       <c r="C4" t="s">
         <v>12</v>
+      </c>
+      <c r="D4">
+        <v>11476372224</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>11476372224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>11476372224</v>
       </c>
     </row>
   </sheetData>
@@ -500,245 +550,119 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>